<commit_message>
Entrega final parcial 2
- Correcciones H-01 (C10/C15 e IOrquestacionAnalitica) y H-02 (dimensión sistema/proceso/producto) en informe y Excel
- Literal A: CUC, bicolumnar y estados R15; literales C/D: deployment simplificado y escenarios QAW
- PDFs exportados y zip de entrega en Entrega/
- .gitignore para .bak_*, .lck y temporales de Office

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0189PyZp59tnBWGhCrS4AwU2
</commit_message>
<xml_diff>
--- a/reques.xlsx
+++ b/reques.xlsx
@@ -641,7 +641,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:R28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
@@ -1811,7 +1811,7 @@
     <mergeCell ref="A22:B22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
@@ -1819,7 +1819,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
@@ -4075,7 +4075,6 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
     <row r="41" ht="23.85" customHeight="1">
       <c r="A41" s="8" t="inlineStr">
         <is>
@@ -4094,7 +4093,6 @@
         <v/>
       </c>
     </row>
-    <row r="43"/>
     <row r="44" ht="25.5" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
@@ -4116,7 +4114,6 @@
         </is>
       </c>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="A48" s="30" t="inlineStr">
         <is>
@@ -4354,7 +4351,7 @@
     <mergeCell ref="A45:K45"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
@@ -4362,7 +4359,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
@@ -5516,7 +5513,7 @@
     <mergeCell ref="E36:H36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
@@ -5524,7 +5521,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AD41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
@@ -7787,7 +7784,7 @@
     <mergeCell ref="A1:AD1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
@@ -7795,9 +7792,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -7807,6 +7804,7 @@
     <col width="42" customWidth="1" min="5" max="6"/>
     <col width="36" customWidth="1" min="7" max="7"/>
     <col width="44" customWidth="1" min="8" max="8"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="21.75" customHeight="1">
@@ -7856,6 +7854,11 @@
           <t>Literal A: CUC y estados (R15)</t>
         </is>
       </c>
+      <c r="I4" s="33" t="inlineStr">
+        <is>
+          <t>Literal C/D: nodo del deployment · escenario QAW</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="57.75" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
@@ -7899,6 +7902,11 @@
           <t>CU-16, CU-17, CU-18; estados del evento (Parte V)</t>
         </is>
       </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>Eventos; Terminal de Campo · QAW-1</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30.75" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -7941,6 +7949,11 @@
           <t>Actor «dispositivo» Terminal de Campo (restricción ergonómica)</t>
         </is>
       </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>Terminal de Campo «SISD» · —</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30.75" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
@@ -7981,6 +7994,11 @@
       <c r="H7" s="9" t="inlineStr">
         <is>
           <t>R3.4 como precondición de CU-01 y CU-06 (bicolumnar)</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>Servidores de seguridad · —</t>
         </is>
       </c>
     </row>
@@ -8027,6 +8045,11 @@
           <t>CU-01, CU-02, CU-03 (bicolumnar de CU-01)</t>
         </is>
       </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Servidores web y de monitoreo · QAW-1</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="44.25" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
@@ -8069,6 +8092,11 @@
           <t>CUC y diagramas de estados en notación UML 2.5</t>
         </is>
       </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>Todos los diagramas en UML 2.5 · —</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="44.25" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -8112,6 +8140,11 @@
           <t>CU-12, CU-14, CU-15</t>
         </is>
       </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>Ingesta; Mensajería; Series de tiempo · QAW-1, QAW-3</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="44.25" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
@@ -8155,6 +8188,11 @@
           <t>CU-06 a CU-11 (bicolumnar de CU-06)</t>
         </is>
       </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>Analítica «MIMD/SIMD»; Topología · QAW-3</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -8197,6 +8235,11 @@
           <t>CU-21</t>
         </is>
       </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>Servidores de seguridad · —</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="44.25" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
@@ -8238,6 +8281,11 @@
       <c r="H13" s="9" t="inlineStr">
         <is>
           <t>CU-04 («extend» de CU-01), CU-05</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>Servidores web y de monitoreo; Topología · QAW-1</t>
         </is>
       </c>
     </row>
@@ -8282,6 +8330,11 @@
       <c r="H14" s="9" t="inlineStr">
         <is>
           <t>CU-19; estados de la sesión (Parte V)</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>Servidores de seguridad · —</t>
         </is>
       </c>
     </row>
@@ -8329,6 +8382,11 @@
           <t>— (RNF: deployment y QAW)</t>
         </is>
       </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>Mensajería y Series de tiempo replicados · QAW-2, QAW-3</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -8369,6 +8427,11 @@
       <c r="H16" s="9" t="inlineStr">
         <is>
           <t>CU-13</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>Clúster de ingesta · QAW-1</t>
         </is>
       </c>
     </row>
@@ -8416,6 +8479,11 @@
           <t>— (RNF: deployment y QAW)</t>
         </is>
       </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>Todos los clústeres «MIMD» · QAW-2</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30.75" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -8458,6 +8526,11 @@
           <t>— (fuera del alcance del CUC de R4/R7)</t>
         </is>
       </c>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>Zona de APIs · —</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="44.25" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
@@ -8499,6 +8572,11 @@
       <c r="H19" s="9" t="inlineStr">
         <is>
           <t>Diagramas de estados del evento y de la sesión (Parte V)</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>— (diagramas de estados, Parte V)</t>
         </is>
       </c>
     </row>
@@ -8508,7 +8586,7 @@
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
@@ -8516,7 +8594,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
@@ -8536,6 +8614,7 @@
     <row r="2">
       <c r="A2" s="6" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4" ht="36" customFormat="1" customHeight="1" s="16">
       <c r="A4" s="33" t="inlineStr">
         <is>
@@ -9055,7 +9134,7 @@
       <c r="E14" s="9" t="inlineStr">
         <is>
           <t>• Construir el mapa georreferenciado de Cali con transformadores y circuitos
-• Calcular el estado de cada elemento (normal, advertencia, corte, sospecha de fraude) desde lecturas y eventos activos
+• Calcular el estado de cada elemento (normal, advertencia, corte, sospecha de fraude) desde lecturas, eventos activos y el último % de pérdidas no técnicas del balance (C15)
 • Aplicar el filtro de zonas cuando se solicita una vista de operador</t>
         </is>
       </c>
@@ -9069,7 +9148,8 @@
           <t>• ICicloVidaEventos (C05 GestorCicloVidaEventos)
 • IConsultaTelemetria (C09 ServicioConsultaTelemetria)
 • ITopologiaRed (C13 CatalogoTopologiaRed)
-• IAutorizacion (C20 AutorizadorAcceso)</t>
+• IAutorizacion (C20 AutorizadorAcceso)
+• IOrquestacionAnalitica (C15 OrquestadorAnaliticaPerdidas)</t>
         </is>
       </c>
       <c r="H14" s="10" t="inlineStr">
@@ -9317,7 +9397,7 @@
         <is>
           <t>• Recibir la solicitud de balance mensual por año, transformador o circuito
 • Particionar el trabajo por transformador y mes
-• Entregar los resultados a la consola</t>
+• Entregar los resultados a la consola y el % de pérdidas al mapa (C10)</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
@@ -9844,7 +9924,7 @@
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
@@ -9852,7 +9932,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
@@ -9870,6 +9950,7 @@
     <row r="2">
       <c r="A2" s="6" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customFormat="1" customHeight="1" s="16">
       <c r="A4" s="33" t="inlineStr">
         <is>
@@ -10288,7 +10369,7 @@
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>ConsolaWebCOD</t>
+          <t>ConsolaWebCOD, ServicioMapaRed</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
@@ -10572,6 +10653,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31" ht="25.5" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
@@ -10586,6 +10668,6 @@
     <mergeCell ref="A31:E31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>